<commit_message>
Update results after re-checking the manual labels
The author re-checked the manual labels blind, using the page content
saved at collection time. Domain-for-sale pages and gambling pages that
had been missed were corrected, and the classifier metrics, robustness
checks and blind verification results were recomputed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/tables_and_figures.xlsx
+++ b/results/tables_and_figures.xlsx
@@ -869,21 +869,21 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>86.3</v>
+        <v>80.2</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>79.3〜91.1</t>
+          <t>72.5〜86.1</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>0.75（36/48）</t>
+          <t>0.69（36/52）</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>0.61〜0.85</t>
+          <t>0.56〜0.80</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -902,29 +902,29 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>89.3</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>82.9〜93.5</t>
+          <t>85.6〜95.2</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>0.90（43/48）</t>
+          <t>0.92（48/52）</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>0.78〜0.95</t>
+          <t>0.82〜0.97</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.84</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>0.016</t>
+          <t>&lt;0.001</t>
         </is>
       </c>
     </row>
@@ -935,29 +935,29 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>90.09999999999999</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>83.8〜94.1</t>
+          <t>86.5〜95.8</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>0.92（44/48）</t>
+          <t>0.94（49/52）</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>0.80〜0.97</t>
+          <t>0.84〜0.98</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.85</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>0.008</t>
+          <t>&lt;0.001</t>
         </is>
       </c>
     </row>
@@ -968,29 +968,29 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>89.3</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>82.9〜93.5</t>
+          <t>85.6〜95.2</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>0.92（44/48）</t>
+          <t>0.94（49/52）</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>0.80〜0.97</t>
+          <t>0.84〜0.98</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.83</v>
+        <v>0.92</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>0.008</t>
+          <t>&lt;0.001</t>
         </is>
       </c>
     </row>
@@ -1001,29 +1001,29 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>90.09999999999999</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>83.8〜94.1</t>
+          <t>86.5〜95.8</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>0.92（44/48）</t>
+          <t>0.94（49/52）</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>0.80〜0.97</t>
+          <t>0.84〜0.98</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.85</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>0.008</t>
+          <t>&lt;0.001</t>
         </is>
       </c>
     </row>
@@ -1034,29 +1034,29 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>86.3</v>
+        <v>87.8</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>79.3〜91.1</t>
+          <t>81.1〜92.3</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>0.83（40/48）</t>
+          <t>0.87（45/52）</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>0.70〜0.91</t>
+          <t>0.75〜0.93</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.82</v>
+        <v>0.92</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>0.289</t>
+          <t>0.022</t>
         </is>
       </c>
     </row>
@@ -1105,22 +1105,22 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>93.59999999999999</v>
+        <v>92.8</v>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>0.78</t>
+          <t>0.80</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>0.39〜0.95</t>
+          <t>0.42〜0.96</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>0.81（17/21）</t>
+          <t>0.90（19/21）</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -1132,7 +1132,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>70.59999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr">
@@ -1142,12 +1142,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>0.30〜0.73</t>
+          <t>0.31〜0.70</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>0.57（13/23）</t>
+          <t>0.61（14/23）</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -1420,7 +1420,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>読込 verify_labels.csv  判定 100件（判断不能 1件）</t>
+          <t>読込 verify_labels_v2_20261018.csv  判定 100件（判断不能 1件）</t>
         </is>
       </c>
     </row>
@@ -1436,14 +1436,14 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  gpt-5.5: abuse判定 21件のうち目視でabuse 17件  適合率 0.81（95%CI 0.60〜0.92）  誤りの内訳 live 2 / non-content 2</t>
+          <t xml:space="preserve">  gpt-5.5: abuse判定 21件のうち目視でabuse 19件  適合率 0.90（95%CI 0.71〜0.97）  誤りの内訳 live 1 / non-content 1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  語彙規則: abuse判定 23件のうち目視でabuse 13件  適合率 0.57（95%CI 0.37〜0.74）  誤りの内訳 live 10 / non-content 0</t>
+          <t xml:space="preserve">  語彙規則: abuse判定 23件のうち目視でabuse 14件  適合率 0.61（95%CI 0.41〜0.78）  誤りの内訳 live 9 / non-content 0</t>
         </is>
       </c>
     </row>
@@ -1457,14 +1457,14 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  gpt-5.5 の推定再現率 17/21.9 = 0.78（abuse判定ありの層の確認済み abuse 17件＋見逃し推定 4.9件）</t>
+          <t xml:space="preserve">  gpt-5.5 の推定再現率 19/23.9 = 0.80（abuse判定ありの層の確認済み abuse 19件＋見逃し推定 4.9件）</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  語彙規則 の推定再現率 13/21.9 = 0.59（abuse判定ありの層の確認済み abuse 17件＋見逃し推定 4.9件）</t>
+          <t xml:space="preserve">  語彙規則 の推定再現率 14/23.9 = 0.59（abuse判定ありの層の確認済み abuse 19件＋見逃し推定 4.9件）</t>
         </is>
       </c>
     </row>
@@ -1480,14 +1480,14 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  gpt-5.5: 正解率 93.6%（abuse判定ありの層 25/29，それ以外の層 65/69，母数 367件）</t>
+          <t xml:space="preserve">  gpt-5.5: 正解率 92.8%（abuse判定ありの層 27/29，それ以外の層 64/69，母数 367件）</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  語彙規則: 正解率 70.6%（abuse判定ありの層 14/29，それ以外の層 50/69，母数 367件）</t>
+          <t xml:space="preserve">  語彙規則: 正解率 69.5%（abuse判定ありの層 15/29，それ以外の層 49/69，母数 367件）</t>
         </is>
       </c>
     </row>
@@ -1510,21 +1510,21 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  [目視で確認したabuse（abuse判定ありの層＋無作為抽出の層）] 新規 8/105=7.6%  既存 8/650=1.2%  OR=6.62  リスク比=6.19  Fisher p=5.3e-04  abuseに占める新規 8/16=50.0%（CI 28〜72%）</t>
+          <t xml:space="preserve">  [目視で確認したabuse（abuse判定ありの層＋無作為抽出の層）] 新規 9/105=8.6%  既存 9/650=1.4%  OR=6.68  リスク比=6.19  Fisher p=2.3e-04  abuseに占める新規 9/18=50.0%（CI 29〜71%）</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  gpt-5.5 の適合率（新規） 8/10</t>
+          <t xml:space="preserve">  gpt-5.5 の適合率（新規） 9/10</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  gpt-5.5 の適合率（既存） 8/10</t>
+          <t xml:space="preserve">  gpt-5.5 の適合率（既存） 9/10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add weighted classifier metrics and additional robustness checks
- Weight the classifier evaluation by the sizes of the sampling strata
  (the 190 labeled pages were stratified by the heuristic classifier),
  with stratified bootstrap confidence intervals.
- Add checks requested in review: sensitivity of the certificate-history
  newness judgment, allocation of missed abuse to existing domains, and
  weighting by the daily number of newly observed domains.
- Exclude labels the author could not settle, and apply Holm's correction
  to the three LLM-vs-heuristic recall comparisons used in the paper.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/tables_and_figures.xlsx
+++ b/results/tables_and_figures.xlsx
@@ -8,13 +8,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参考_流量と被覆率" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表1_閾値と既存の割合" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表2_分類器の性能" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表3_新規既存別の内容" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表3補足_目視確認" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表3補足_頑健性" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="図1_元データ" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="図2_元データ" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参考_追加の確認" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表1_閾値と既存の割合" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表2_分類器の性能" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表2補足_重み付け" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表3_新規既存別の内容" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表3補足_目視確認" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表3補足_頑健性" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="図1_元データ" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="図2_元データ" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -626,7 +628,412 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40.40000000000001" customWidth="1" min="1" max="1"/>
+    <col width="38.8" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>先行日数（日）</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>サービス数</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2–14</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>15–30</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>31–60</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>61–120</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>121–365</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>計画（過去24か月のShow HN, 重複除く）</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>初回証明書日を取得できた件数</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>先行率(%)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>99.90000000000001</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>先行率の95%CI(%)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>99.3〜100.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>新規ローンチ帯（先行0〜365日）</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>先行日数 中央値</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>先行日数 第1・第3四分位</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>7・107</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>30日以上(%)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>90日以上(%)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>0〜1日（件, %）</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>60, 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>RDAP登録日を取得できた件数</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>675（81.5%）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>新規ローンチ帯で登録日もある件数</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>登録→初回証明書 中央値（日）</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>登録→初回証明書 7日以内(%)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>登録から1年以内に告知（件, %）</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>446, 66.1（CI 62.4〜69.5）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>その登録→告知 中央値・第1・第3四分位</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>36・9・110</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>新規判定の感度，見逃しを既存に寄せた場合，収集日による重み付け（paper_tools/extra_checks.py）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2">
+        <f>=== 1. 証明書履歴による新規判定（基準：RDAP の登録日，閾値120日） ====</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  対象 162件（初観測日: {'2026-08-18': 10, '2026-08-19': 30, '2026-09-03': 122}）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  感度（RDAPで新規のうち証明書履歴でも新規）: 15/20 = 0.750（95%CI 0.53〜0.89）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  特異度（RDAPで既存のうち証明書履歴でも既存）: 142/142 = 1.000（95%CI 0.97〜1.00）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  陽性的中率（証明書履歴で新規のうちRDAPでも新規）: 15/15 = 1.000（95%CI 0.80〜1.00）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  陰性的中率: 142/147 = 0.966（95%CI 0.92〜0.99）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <f>=== 2. 目視で確認した abuse：見逃しを既存ドメインに寄せた場合 ====</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  確認済み abuse：新規 8/105  既存 8/650</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  どちらの分類器も abuse としなかった内容のあるページ 338件（新規 35，既存 217，登録日不明 86）  見逃しの割合 1.4%（95%CI 0.3〜7.8%）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  見逃しを層の件数に応じて配分（点推定）: 新規 8.5/105  既存 11.1/650 → 四捨五入 9/105=8.6% と 11/650=1.7%  OR=5.45  RR=5.06  Fisher p=6.2e-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  見逃しをすべて既存に寄せる（点推定）: 新規 8.0/105  既存 11.7/650 → 四捨五入 8/105=7.6% と 12/650=1.8%  OR=4.38  RR=4.13  Fisher p=3.2e-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  見逃しをすべて既存に寄せる（95%CIの上限）: 新規 8.0/105  既存 27.6/650 → 四捨五入 8/105=7.6% と 28/650=4.3%  OR=1.83  RR=1.77  Fisher p=1.4e-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2">
+        <f>=== 3. 収集日ごとの新規観測ドメイン数で重み付け ====</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  収集日 68日（新規観測数が不明な日 0日は除く）  重み = その日の新規観測数 / その日の標本数</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  既存の割合：重みなし 86.1%  重み付き 85.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  gpt-5.5 の abuse の割合：新規 9.9%  既存 1.9%  リスク比 5.25  オッズ比 5.72（重み付き）</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -807,7 +1214,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -869,21 +1276,21 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>80.2</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>72.5〜86.1</t>
+          <t>74.3〜87.6</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>0.69（36/52）</t>
+          <t>0.73（35/48）</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>0.56〜0.80</t>
+          <t>0.59〜0.83</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -902,21 +1309,21 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>91.59999999999999</v>
+        <v>91.3</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>85.6〜95.2</t>
+          <t>85.2〜95.1</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>0.92（48/52）</t>
+          <t>0.92（44/48）</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>0.82〜0.97</t>
+          <t>0.80〜0.97</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -924,7 +1331,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;0.001</t>
+          <t>0.004</t>
         </is>
       </c>
     </row>
@@ -935,21 +1342,21 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>92.40000000000001</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>86.5〜95.8</t>
+          <t>86.1〜95.7</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>0.94（49/52）</t>
+          <t>0.94（45/48）</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>0.84〜0.98</t>
+          <t>0.83〜0.98</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -957,7 +1364,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;0.001</t>
+          <t>0.002</t>
         </is>
       </c>
     </row>
@@ -968,21 +1375,21 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>91.59999999999999</v>
+        <v>91.3</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>85.6〜95.2</t>
+          <t>85.2〜95.1</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>0.94（49/52）</t>
+          <t>0.94（45/48）</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>0.84〜0.98</t>
+          <t>0.83〜0.98</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -990,7 +1397,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;0.001</t>
+          <t>0.002</t>
         </is>
       </c>
     </row>
@@ -1001,21 +1408,21 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>92.40000000000001</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>86.5〜95.8</t>
+          <t>86.1〜95.7</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>0.94（49/52）</t>
+          <t>0.94（45/48）</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>0.84〜0.98</t>
+          <t>0.83〜0.98</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -1023,7 +1430,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;0.001</t>
+          <t>0.002</t>
         </is>
       </c>
     </row>
@@ -1034,29 +1441,29 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>87.8</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>81.1〜92.3</t>
+          <t>80.5〜92.1</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>0.87（45/52）</t>
+          <t>0.85（41/48）</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>0.75〜0.93</t>
+          <t>0.73〜0.93</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.92</v>
+        <v>0.91</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>0.022</t>
+          <t>0.109</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1479,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>【無作為標本の目視確認（100件，盲検）】</t>
+          <t>【無作為標本の目視確認（100件，盲検。判定を確定できなかったものを除く）】</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1105,22 +1512,22 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>92.8</v>
+        <v>92.7</v>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>0.78</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>0.42〜0.96</t>
+          <t>0.39〜0.95</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>0.90（19/21）</t>
+          <t>0.89（17/19）</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -1132,22 +1539,22 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>69.5</v>
+        <v>69.3</v>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>0.59</t>
+          <t>0.55</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>0.31〜0.70</t>
+          <t>0.28〜0.67</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>0.61（14/23）</t>
+          <t>0.57（12/21）</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -1155,7 +1562,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>※内容のあるページ367件で層の大きさに応じて重み付け。再現率は見逃しの割合（69件中1件）とその95%CIから推定</t>
+          <t>※本文のあるページ365件で層の大きさに応じて重み付け。再現率は見逃しの割合（69件中1件）とその95%CIから推定</t>
         </is>
       </c>
       <c r="B12" s="2" t="n"/>
@@ -1174,7 +1581,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>正解付き到達ページ131件。gpt-5.5の3回の試行間一致 99.2〜100%，Fleissのκ=0.990</t>
+          <t>正解付きの本文のあるページ127件（判定を確定できなかったものを除く）。gpt-5.5の3回の試行間一致 99.2〜100%，Fleissのκ=0.990</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1590,115 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>正解190件の層化を母集団の層の大きさで重み付けした推定（paper_tools/weighted_gold.py）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>母集団3,336件の層（ヒューリスティック分類器の3分類）: {'non-content': 2395, 'live': 781, 'abuse': 160}  抽出: {'live': 90, 'non-content': 60, 'abuse': 40}  重み: live=8.68, non-content=39.92, abuse=4.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>評価の対象: 内容のあるページのうち判断できた 127 件</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>分類器: 重み付き正解率 / abuse再現率 / abuse適合率（95%CI，層別ブートストラップ2,000回）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ヒューリスティック: 正解率 75.6%（65.2〜86.0）  再現率 0.44（0.31〜0.66）  適合率 0.92（0.82〜1.00）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  gpt-5.3-codex-spark: 正解率 91.1%（85.3〜95.7）  再現率 0.89（0.76〜0.98）  適合率 0.93（0.83〜1.00）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  gpt-5.5（a）: 正解率 91.9%（86.2〜96.5）  再現率 0.92（0.81〜1.00）  適合率 0.93（0.84〜1.00）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  gpt-5.5（b）: 正解率 91.1%（85.1〜95.9）  再現率 0.92（0.81〜1.00）  適合率 0.91（0.80〜0.99）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  gpt-5.5（c）: 正解率 91.9%（86.2〜96.5）  再現率 0.92（0.81〜1.00）  適合率 0.93（0.84〜1.00）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Qwen2.5-7B-Instruct: 正解率 87.7%（81.5〜93.4）  再現率 0.84（0.70〜0.95）  適合率 0.90（0.78〜0.99）</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  再現率の差（gpt-5.3-codex-spark − ヒューリスティック）: +0.45（95%CI +0.20〜+0.61）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  再現率の差（gpt-5.5（a） − ヒューリスティック）: +0.47（95%CI +0.23〜+0.64）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  再現率の差（Qwen2.5-7B-Instruct − ヒューリスティック）: +0.39（95%CI +0.13〜+0.57）</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1398,7 +1913,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1420,7 +1935,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>読込 verify_labels_v2_20261018.csv  判定 100件（判断不能 1件）</t>
+          <t>読込 verify_labels_v2_20261018.csv  判定 100件（判断不能 3件）</t>
         </is>
       </c>
     </row>
@@ -1436,14 +1951,14 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  gpt-5.5: abuse判定 21件のうち目視でabuse 19件  適合率 0.90（95%CI 0.71〜0.97）  誤りの内訳 live 1 / non-content 1</t>
+          <t xml:space="preserve">  gpt-5.5: abuse判定 19件のうち目視でabuse 17件  適合率 0.89（95%CI 0.69〜0.97）  誤りの内訳 live 1 / non-content 1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  語彙規則: abuse判定 23件のうち目視でabuse 14件  適合率 0.61（95%CI 0.41〜0.78）  誤りの内訳 live 9 / non-content 0</t>
+          <t xml:space="preserve">  語彙規則: abuse判定 21件のうち目視でabuse 12件  適合率 0.57（95%CI 0.37〜0.76）  誤りの内訳 live 9 / non-content 0</t>
         </is>
       </c>
     </row>
@@ -1457,14 +1972,14 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  gpt-5.5 の推定再現率 19/23.9 = 0.80（abuse判定ありの層の確認済み abuse 19件＋見逃し推定 4.9件）</t>
+          <t xml:space="preserve">  gpt-5.5 の推定再現率 17/21.9 = 0.78（abuse判定ありの層の確認済み abuse 17件＋見逃し推定 4.9件）</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  語彙規則 の推定再現率 14/23.9 = 0.59（abuse判定ありの層の確認済み abuse 19件＋見逃し推定 4.9件）</t>
+          <t xml:space="preserve">  語彙規則 の推定再現率 12/21.9 = 0.55（abuse判定ありの層の確認済み abuse 17件＋見逃し推定 4.9件）</t>
         </is>
       </c>
     </row>
@@ -1480,14 +1995,14 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  gpt-5.5: 正解率 92.8%（abuse判定ありの層 27/29，それ以外の層 64/69，母数 367件）</t>
+          <t xml:space="preserve">  gpt-5.5: 正解率 92.7%（abuse判定ありの層 25/27，それ以外の層 64/69，母数 365件）</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  語彙規則: 正解率 69.5%（abuse判定ありの層 15/29，それ以外の層 49/69，母数 367件）</t>
+          <t xml:space="preserve">  語彙規則: 正解率 69.3%（abuse判定ありの層 13/27，それ以外の層 49/69，母数 365件）</t>
         </is>
       </c>
     </row>
@@ -1510,21 +2025,21 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  [目視で確認したabuse（abuse判定ありの層＋無作為抽出の層）] 新規 9/105=8.6%  既存 9/650=1.4%  OR=6.68  リスク比=6.19  Fisher p=2.3e-04  abuseに占める新規 9/18=50.0%（CI 29〜71%）</t>
+          <t xml:space="preserve">  [目視で確認したabuse（abuse判定ありの層＋無作為抽出の層）] 新規 8/105=7.6%  既存 8/650=1.2%  OR=6.62  リスク比=6.19  Fisher p=5.3e-04  abuseに占める新規 8/16=50.0%（CI 28〜72%）</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  gpt-5.5 の適合率（新規） 9/10</t>
+          <t xml:space="preserve">  gpt-5.5 の適合率（新規） 8/9</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  gpt-5.5 の適合率（既存） 9/10</t>
+          <t xml:space="preserve">  gpt-5.5 の適合率（既存） 8/9</t>
         </is>
       </c>
     </row>
@@ -1533,7 +2048,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2138,7 +2653,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RDAP登録日を取得できた755件。「新規の割合」は標本に占める新規ドメインの割合，「abuseに占める新規」はabuseと分類されたドメインのうち新規ドメインの割合</t>
+          <t>RDAP登録日を取得できた755件。「新規の割合」は登録日を取得できたドメインに占める新規ドメインの割合，「abuseに占める新規」はabuseと分類されたドメインのうち新規ドメインの割合</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2662,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2235,270 +2750,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40.40000000000001" customWidth="1" min="1" max="1"/>
-    <col width="38.8" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>先行日数（日）</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>サービス数</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>0–1</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2–14</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>15–30</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>31–60</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>61–120</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>121–365</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>計画（過去24か月のShow HN, 重複除く）</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>828</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>初回証明書日を取得できた件数</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>827</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>先行率(%)</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>99.90000000000001</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>先行率の95%CI(%)</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>99.3〜100.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>新規ローンチ帯（先行0〜365日）</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>先行日数 中央値</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>先行日数 第1・第3四分位</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>7・107</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>30日以上(%)</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>90日以上(%)</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>0〜1日（件, %）</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>60, 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>RDAP登録日を取得できた件数</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>675（81.5%）</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>新規ローンチ帯で登録日もある件数</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>登録→初回証明書 中央値（日）</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>登録→初回証明書 7日以内(%)</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>登録から1年以内に告知（件, %）</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>446, 66.1（CI 62.4〜69.5）</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>その登録→告知 中央値・第1・第3四分位</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>36・9・110</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>